<commit_message>
Updated unit tests with dashboard changes
</commit_message>
<xml_diff>
--- a/example_cramino_dashboard.xlsx
+++ b/example_cramino_dashboard.xlsx
@@ -19,8 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mean length plot" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Median identity plot" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mean identity plot" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Median mapping Q score plot" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mean mapping Q score plot" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Median identity Q score plot" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mean identity Q score plot" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yield (Gb) vs. med. idy" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="N50 (kb) vs. med. idy" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pct. total vs. med. idy" sheetId="18" state="visible" r:id="rId18"/>
@@ -1628,7 +1628,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Median mapping Q score</t>
+          <t>Median identity Q score</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1656,7 +1656,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mean mapping Q score</t>
+          <t>Mean identity Q score</t>
         </is>
       </c>
       <c r="B15" t="n">

</xml_diff>